<commit_message>
add l2tlb function dercription
</commit_message>
<xml_diff>
--- a/doc/l1dtlb_uvm_audit/L1DTLB_TRISTAN_IP_Hardware_tp_V1.xlsx
+++ b/doc/l1dtlb_uvm_audit/L1DTLB_TRISTAN_IP_Hardware_tp_V1.xlsx
@@ -654,15 +654,15 @@
     <t xml:space="preserve">credit上下界和守恒</t>
   </si>
   <si>
-    <t xml:space="preserve">reset、连续发request、credit return、request+return同拍，覆盖credit=0</t>
+    <t xml:space="preserve">reset、连续发request、credit return、credit&gt;0时request+return同拍，覆盖credit=0且return同拍</t>
   </si>
   <si>
     <t xml:space="preserve">`test_mmu_l1dtlb_dtlb_credit_001`, `_002`, `test_mmu_l1dtlb_dtlb_credit_bound_001`</t>
   </si>
   <si>
     <t xml:space="preserve">Purpose: credit上下界和守恒
-Stimuli: reset、连续发request、credit return、request+return同拍，覆盖credit=0
-Expected: credit初值为DTLB专用ReqQ深度；只被request消耗、return归还；同拍request+return计数不变；credit=0且同拍return允许发一个request</t>
+Stimuli: reset、连续发request、credit return、credit&gt;0时request+return同拍，覆盖credit=0且return同拍
+Expected: credit初值为DTLB专用ReqQ深度；只被request消耗、return归还；credit&gt;0时同拍request+return计数不变；credit=0且同拍return不得当拍发request，return只让下一拍credit可用</t>
   </si>
   <si>
     <t xml:space="preserve">Criteria (PASS/FAIL): scheduler credit probe或SVA，request fire条件与credit一致. A UVM_ERROR, SVA failure, scoreboard mismatch, or missing required coverage bin fails this item.</t>

</xml_diff>